<commit_message>
THIS IS WHERE WE HOLD THEM. THIS IS WHERE WE FIGHT. THIS IS WHERE THEY DIE.
Final Safeguard before going for results.
Have made one final batch of CMs, and also I'm now using 7 CMs per run instead of 8. End of Issue #40
I'm one with the Force and the Force is with me...
</commit_message>
<xml_diff>
--- a/Thesis/H2S AEGL.xlsx
+++ b/Thesis/H2S AEGL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gavin\Documents\GitHub\evac\Thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91F0C28-DB12-435A-A317-AA3F75459C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FFB0C2-A759-4219-869C-C6E1BC23B2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
   </bookViews>
   <sheets>
     <sheet name="New_AEGL" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="80">
   <si>
     <t>Fit Smell</t>
   </si>
@@ -144,9 +144,6 @@
     <t>ppm*255/1000</t>
   </si>
   <si>
-    <t>afafaf</t>
-  </si>
-  <si>
     <t>Duration</t>
   </si>
   <si>
@@ -268,6 +265,18 @@
   </si>
   <si>
     <t>c(t)=8.5*t^(-0,227)</t>
+  </si>
+  <si>
+    <t>AFAFAF</t>
+  </si>
+  <si>
+    <t>3F3F3F</t>
+  </si>
+  <si>
+    <t>2E2E2E</t>
+  </si>
+  <si>
+    <t>2B2B2B</t>
   </si>
 </sst>
 </file>
@@ -334,11 +343,11 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="45"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2627,7 +2636,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
@@ -2637,8 +2646,8 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
-        <v>73</v>
+      <c r="A2" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="B2" s="2">
         <v>493.13517353857929</v>
@@ -2667,7 +2676,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="7"/>
+      <c r="A3" s="8"/>
       <c r="B3" s="2">
         <v>439.14335359378231</v>
       </c>
@@ -2680,7 +2689,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
+      <c r="A4" s="8"/>
       <c r="B4" s="2">
         <v>375.20835895751202</v>
       </c>
@@ -2693,7 +2702,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="7"/>
+      <c r="A5" s="8"/>
       <c r="B5" s="2">
         <v>342.21558912436569</v>
       </c>
@@ -2706,7 +2715,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
+      <c r="A6" s="8"/>
       <c r="B6" s="2">
         <v>292.39233283217675</v>
       </c>
@@ -2733,8 +2742,8 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
-        <v>74</v>
+      <c r="A10" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="B10" s="2">
         <v>232.86938750432913</v>
@@ -2759,7 +2768,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
+      <c r="A11" s="8"/>
       <c r="B11" s="2">
         <v>207.37325030817499</v>
       </c>
@@ -2768,7 +2777,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
+      <c r="A12" s="8"/>
       <c r="B12" s="2">
         <v>177.18172506326957</v>
       </c>
@@ -2777,7 +2786,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
+      <c r="A13" s="8"/>
       <c r="B13" s="2">
         <v>161.60180597539491</v>
       </c>
@@ -2786,7 +2795,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
+      <c r="A14" s="8"/>
       <c r="B14" s="2">
         <v>138.07415717075011</v>
       </c>
@@ -2809,8 +2818,8 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
-        <v>75</v>
+      <c r="A18" s="8" t="s">
+        <v>74</v>
       </c>
       <c r="B18" s="2">
         <v>164.37839117952643</v>
@@ -2835,7 +2844,7 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="7"/>
+      <c r="A19" s="8"/>
       <c r="B19" s="2">
         <v>146.3811178645941</v>
       </c>
@@ -2844,7 +2853,7 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="7"/>
+      <c r="A20" s="8"/>
       <c r="B20" s="2">
         <v>125.06945298583734</v>
       </c>
@@ -2853,7 +2862,7 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="7"/>
+      <c r="A21" s="8"/>
       <c r="B21" s="2">
         <v>114.07186304145523</v>
       </c>
@@ -2862,7 +2871,7 @@
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="7"/>
+      <c r="A22" s="8"/>
       <c r="B22" s="2">
         <v>97.464110944058902</v>
       </c>
@@ -2879,8 +2888,8 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
-        <v>76</v>
+      <c r="A26" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="B26" s="3">
         <v>2.3286938750432911</v>
@@ -2905,7 +2914,7 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="7"/>
+      <c r="A27" s="8"/>
       <c r="B27" s="3">
         <v>2.0737325030817497</v>
       </c>
@@ -2914,7 +2923,7 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="7"/>
+      <c r="A28" s="8"/>
       <c r="B28" s="3">
         <v>1.7718172506326957</v>
       </c>
@@ -2923,7 +2932,7 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="7"/>
+      <c r="A29" s="8"/>
       <c r="B29" s="3">
         <v>1.6160180597539491</v>
       </c>
@@ -2932,7 +2941,7 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="7"/>
+      <c r="A30" s="8"/>
       <c r="B30" s="3">
         <v>1.3807415717075011</v>
       </c>
@@ -2940,10 +2949,10 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="35" spans="1:3" s="8" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="35" spans="1:3" s="7" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>3</v>
@@ -2953,8 +2962,8 @@
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="7" t="s">
-        <v>73</v>
+      <c r="A37" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="B37" s="2">
         <f>1800*C37^(-0.227)</f>
@@ -2965,7 +2974,7 @@
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="7"/>
+      <c r="A38" s="8"/>
       <c r="B38" s="2">
         <f t="shared" ref="B38:B41" si="1">1800*C38^(-0.227)</f>
         <v>493.13517353857929</v>
@@ -2975,7 +2984,7 @@
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="7"/>
+      <c r="A39" s="8"/>
       <c r="B39" s="2">
         <f t="shared" si="1"/>
         <v>443.23162915052404</v>
@@ -2985,7 +2994,7 @@
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="7"/>
+      <c r="A40" s="8"/>
       <c r="B40" s="2">
         <f t="shared" si="1"/>
         <v>384.29032922710877</v>
@@ -2995,7 +3004,7 @@
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="7"/>
+      <c r="A41" s="8"/>
       <c r="B41" s="2">
         <f t="shared" si="1"/>
         <v>328.34140062136413</v>
@@ -3019,8 +3028,8 @@
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="7" t="s">
-        <v>74</v>
+      <c r="A45" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="B45" s="2">
         <f>850*C45^(-0.227)</f>
@@ -3031,7 +3040,7 @@
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="7"/>
+      <c r="A46" s="8"/>
       <c r="B46" s="2">
         <f t="shared" ref="B46:B49" si="2">850*C46^(-0.227)</f>
         <v>232.86938750432913</v>
@@ -3041,7 +3050,7 @@
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="7"/>
+      <c r="A47" s="8"/>
       <c r="B47" s="2">
         <f t="shared" si="2"/>
         <v>209.30382487663636</v>
@@ -3051,7 +3060,7 @@
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="7"/>
+      <c r="A48" s="8"/>
       <c r="B48" s="2">
         <f t="shared" si="2"/>
         <v>181.47043324613469</v>
@@ -3061,7 +3070,7 @@
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="7"/>
+      <c r="A49" s="8"/>
       <c r="B49" s="2">
         <f t="shared" si="2"/>
         <v>155.05010584897749</v>
@@ -3085,8 +3094,8 @@
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="7" t="s">
-        <v>75</v>
+      <c r="A53" s="8" t="s">
+        <v>74</v>
       </c>
       <c r="B53" s="2">
         <f>600*C53^(-0.227)</f>
@@ -3097,7 +3106,7 @@
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="7"/>
+      <c r="A54" s="8"/>
       <c r="B54" s="2">
         <f t="shared" ref="B54:B57" si="3">600*C54^(-0.227)</f>
         <v>164.37839117952643</v>
@@ -3107,7 +3116,7 @@
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="7"/>
+      <c r="A55" s="8"/>
       <c r="B55" s="2">
         <f t="shared" si="3"/>
         <v>147.74387638350802</v>
@@ -3117,7 +3126,7 @@
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="7"/>
+      <c r="A56" s="8"/>
       <c r="B56" s="2">
         <f t="shared" si="3"/>
         <v>128.09677640903624</v>
@@ -3127,7 +3136,7 @@
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="7"/>
+      <c r="A57" s="8"/>
       <c r="B57" s="2">
         <f t="shared" si="3"/>
         <v>109.44713354045471</v>
@@ -3145,8 +3154,8 @@
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="7" t="s">
-        <v>76</v>
+      <c r="A61" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="B61" s="2">
         <f>8.5*C61^(-0.227)</f>
@@ -3157,7 +3166,7 @@
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="7"/>
+      <c r="A62" s="8"/>
       <c r="B62" s="2">
         <f t="shared" ref="B62:B65" si="4">8.5*C62^(-0.227)</f>
         <v>2.3286938750432911</v>
@@ -3167,7 +3176,7 @@
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="7"/>
+      <c r="A63" s="8"/>
       <c r="B63" s="2">
         <f t="shared" si="4"/>
         <v>2.0930382487663635</v>
@@ -3177,7 +3186,7 @@
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="7"/>
+      <c r="A64" s="8"/>
       <c r="B64" s="2">
         <f t="shared" si="4"/>
         <v>1.8147043324613468</v>
@@ -3187,7 +3196,7 @@
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="7"/>
+      <c r="A65" s="8"/>
       <c r="B65" s="2">
         <f t="shared" si="4"/>
         <v>1.5505010584897752</v>
@@ -3213,10 +3222,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D976B459-1B7D-4296-8012-F11251EFF08E}">
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.3984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.09765625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
@@ -3235,22 +3245,22 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" t="s">
         <v>57</v>
       </c>
-      <c r="F1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G1" t="s">
-        <v>58</v>
-      </c>
       <c r="I1" t="s">
+        <v>60</v>
+      </c>
+      <c r="J1" t="s">
         <v>61</v>
-      </c>
-      <c r="J1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -3387,6 +3397,9 @@
       <c r="C8" t="s">
         <v>33</v>
       </c>
+      <c r="D8" t="s">
+        <v>57</v>
+      </c>
       <c r="E8" t="s">
         <v>34</v>
       </c>
@@ -3404,15 +3417,15 @@
       <c r="A9" s="4">
         <v>0.317</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="5">
         <f>328.71*A9^(-0.641)</f>
         <v>686.48954787651837</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="5">
         <v>9.3718832874999976</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="E9" s="5">
         <v>175.05483470851217</v>
@@ -3433,11 +3446,11 @@
       <c r="A10" s="4">
         <v>0.63400000000000001</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="5">
         <f t="shared" ref="B10:B18" si="6">328.71*A10^(-0.641)</f>
         <v>440.22398628267081</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="5">
         <v>47.789973149999994</v>
       </c>
       <c r="D10">
@@ -3462,11 +3475,11 @@
       <c r="A11" s="4">
         <v>0.95099999999999996</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="5">
         <f t="shared" si="6"/>
         <v>339.46828397332285</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="5">
         <v>85.12026958749999</v>
       </c>
       <c r="D11">
@@ -3491,12 +3504,15 @@
       <c r="A12" s="4">
         <v>1.268</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="5">
         <f t="shared" si="6"/>
         <v>282.30168791071554</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="5">
         <v>121.36277259999999</v>
+      </c>
+      <c r="D12">
+        <v>484848</v>
       </c>
       <c r="E12" s="5">
         <v>71.986930417232458</v>
@@ -3517,12 +3533,15 @@
       <c r="A13" s="4">
         <v>1.585</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="5">
         <f t="shared" si="6"/>
         <v>244.67756877690817</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="5">
         <v>156.51748218749998</v>
+      </c>
+      <c r="D13" t="s">
+        <v>77</v>
       </c>
       <c r="E13" s="5">
         <v>62.392780038111582</v>
@@ -3543,12 +3562,15 @@
       <c r="A14" s="4">
         <v>1.9019999999999999</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="5">
         <f t="shared" si="6"/>
         <v>217.69024983633781</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="5">
         <v>190.58439835000001</v>
+      </c>
+      <c r="D14">
+        <v>383838</v>
       </c>
       <c r="E14" s="5">
         <v>55.511013708266148</v>
@@ -3569,12 +3591,15 @@
       <c r="A15" s="4">
         <v>2.2189999999999999</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="5">
         <f>328.71*A15^(-0.641)</f>
         <v>197.20870699513659</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="5">
         <v>223.56352108749996</v>
+      </c>
+      <c r="D15">
+        <v>323232</v>
       </c>
       <c r="E15" s="5">
         <v>50.288220283759827</v>
@@ -3595,12 +3620,15 @@
       <c r="A16" s="4">
         <v>2.536</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="5">
         <f t="shared" si="6"/>
         <v>181.03112388352878</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="5">
         <v>255.45485039999994</v>
+      </c>
+      <c r="D16" t="s">
+        <v>78</v>
       </c>
       <c r="E16" s="5">
         <v>46.162936590299843</v>
@@ -3621,12 +3649,15 @@
       <c r="A17" s="4">
         <v>2.8530000000000002</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="5">
         <f t="shared" si="6"/>
         <v>167.86667208591064</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="5">
         <v>286.2583862875</v>
+      </c>
+      <c r="D17" t="s">
+        <v>79</v>
       </c>
       <c r="E17" s="5">
         <v>42.806001381907215</v>
@@ -3647,12 +3678,15 @@
       <c r="A18">
         <v>3.17</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="5">
         <f t="shared" si="6"/>
         <v>156.90396891563105</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="5">
         <v>315.97412874999998</v>
+      </c>
+      <c r="D18">
+        <v>282828</v>
       </c>
       <c r="E18" s="5">
         <v>40.010512073485913</v>
@@ -3680,19 +3714,19 @@
         <v>19</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H23" t="s">
         <v>7</v>
       </c>
       <c r="I23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
@@ -3714,7 +3748,7 @@
         <v>87.527417354256087</v>
       </c>
       <c r="G24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H24">
         <v>0</v>
@@ -3739,13 +3773,13 @@
         <v>56.128558251040531</v>
       </c>
       <c r="G25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H25" s="5">
         <v>87.527417354256087</v>
       </c>
       <c r="I25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
@@ -3767,13 +3801,13 @@
         <v>43.282206206598659</v>
       </c>
       <c r="G26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H26" s="5">
         <v>56.128558251040531</v>
       </c>
       <c r="I26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
@@ -3795,13 +3829,13 @@
         <v>35.993465208616229</v>
       </c>
       <c r="G27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H27" s="5">
         <v>43.282206206598659</v>
       </c>
       <c r="I27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
@@ -3823,13 +3857,13 @@
         <v>31.196390019055791</v>
       </c>
       <c r="G28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H28" s="5">
         <v>40.417499999999997</v>
       </c>
       <c r="I28" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
@@ -3851,13 +3885,13 @@
         <v>27.755506854133074</v>
       </c>
       <c r="G29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H29" s="5">
         <v>35.827500000000001</v>
       </c>
       <c r="I29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
@@ -3879,13 +3913,13 @@
         <v>25.144110141879914</v>
       </c>
       <c r="G30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H30" s="5">
         <v>25.5</v>
       </c>
       <c r="I30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
@@ -3907,13 +3941,13 @@
         <v>23.081468295149921</v>
       </c>
       <c r="G31" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H31" s="5">
         <v>20.91</v>
       </c>
       <c r="I31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
@@ -3956,13 +3990,17 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B36">
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="E36">
+        <f>A9*1000</f>
+        <v>317</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -3970,40 +4008,56 @@
         <v>3600</v>
       </c>
       <c r="C37" t="s">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="E37">
+        <f t="shared" ref="E37:E45" si="10">A10*1000</f>
+        <v>634</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B38">
         <v>263</v>
       </c>
       <c r="C38" t="s">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="E38">
+        <f t="shared" si="10"/>
+        <v>951</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39" s="4">
         <v>16.4375</v>
       </c>
       <c r="C39" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="E39">
+        <f t="shared" si="10"/>
+        <v>1268</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B40" s="4">
         <v>0.12656875000000001</v>
       </c>
       <c r="C40" t="s">
-        <v>45</v>
+        <v>44</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="10"/>
+        <v>1585</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -4011,7 +4065,11 @@
         <v>126.56875000000001</v>
       </c>
       <c r="C41" t="s">
-        <v>46</v>
+        <v>45</v>
+      </c>
+      <c r="E41">
+        <f t="shared" si="10"/>
+        <v>1902</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -4019,7 +4077,11 @@
         <v>3.5157986111111116E-2</v>
       </c>
       <c r="C42" t="s">
-        <v>44</v>
+        <v>43</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="10"/>
+        <v>2219</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -4027,7 +4089,23 @@
         <v>35157.986111111117</v>
       </c>
       <c r="C43" t="s">
-        <v>47</v>
+        <v>46</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="10"/>
+        <v>2536</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E44">
+        <f t="shared" si="10"/>
+        <v>2853</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E45">
+        <f t="shared" si="10"/>
+        <v>3170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>